<commit_message>
Fix drawing XML tag order in template to prevent Excel repair error
</commit_message>
<xml_diff>
--- a/Daily_Logs_&Voyage.xlsx
+++ b/Daily_Logs_&Voyage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrian\Documents\Equipment Accountability App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A148B5C-6F95-46AF-BCAA-A91DAC35B707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9C13E2-5A98-43BC-A027-687549C5F9AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,6 +426,9 @@
     <xf numFmtId="4" fontId="1" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -441,9 +444,6 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="1" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -687,7 +687,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1711,16 +1711,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>40821</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>27214</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>127906</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>92528</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>789214</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>176892</xdr:rowOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>81642</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1752,16 +1752,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>190337</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>76037</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>598714</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>176892</xdr:rowOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>476794</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>70212</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1955,7 +1955,7 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1973,55 +1973,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
       <c r="N1" s="9"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
       <c r="N2" s="8"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
     </row>
     <row r="4" spans="1:14" s="6" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -2066,7 +2066,7 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="32">
+      <c r="A5" s="33">
         <v>1</v>
       </c>
       <c r="B5" s="24"/>
@@ -2083,7 +2083,7 @@
       <c r="M5" s="24"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="33"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
       <c r="D6" s="28"/>
@@ -2098,7 +2098,7 @@
       <c r="M6" s="24"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="32">
+      <c r="A7" s="33">
         <v>2</v>
       </c>
       <c r="B7" s="24"/>
@@ -2115,7 +2115,7 @@
       <c r="M7" s="24"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="33"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="27"/>
       <c r="C8" s="27"/>
       <c r="D8" s="28"/>
@@ -2130,7 +2130,7 @@
       <c r="M8" s="24"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="32">
+      <c r="A9" s="33">
         <v>3</v>
       </c>
       <c r="B9" s="24"/>
@@ -2147,7 +2147,7 @@
       <c r="M9" s="24"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="33"/>
+      <c r="A10" s="34"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="28"/>
@@ -2162,7 +2162,7 @@
       <c r="M10" s="24"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="32">
+      <c r="A11" s="33">
         <v>4</v>
       </c>
       <c r="B11" s="24"/>
@@ -2179,7 +2179,7 @@
       <c r="M11" s="24"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="33"/>
+      <c r="A12" s="34"/>
       <c r="B12" s="27"/>
       <c r="C12" s="27"/>
       <c r="D12" s="28"/>
@@ -2194,7 +2194,7 @@
       <c r="M12" s="24"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="32">
+      <c r="A13" s="33">
         <v>5</v>
       </c>
       <c r="B13" s="24"/>
@@ -2211,7 +2211,7 @@
       <c r="M13" s="24"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="33"/>
+      <c r="A14" s="34"/>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
       <c r="D14" s="28"/>
@@ -2226,7 +2226,7 @@
       <c r="M14" s="24"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="32">
+      <c r="A15" s="33">
         <v>6</v>
       </c>
       <c r="B15" s="24"/>
@@ -2243,7 +2243,7 @@
       <c r="M15" s="24"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
+      <c r="A16" s="34"/>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
       <c r="D16" s="28"/>
@@ -2258,7 +2258,7 @@
       <c r="M16" s="24"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="32">
+      <c r="A17" s="33">
         <v>7</v>
       </c>
       <c r="B17" s="24"/>
@@ -2275,7 +2275,7 @@
       <c r="M17" s="24"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="33"/>
+      <c r="A18" s="34"/>
       <c r="B18" s="27"/>
       <c r="C18" s="27"/>
       <c r="D18" s="28"/>
@@ -2290,7 +2290,7 @@
       <c r="M18" s="24"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="32">
+      <c r="A19" s="33">
         <v>8</v>
       </c>
       <c r="B19" s="24"/>
@@ -2307,7 +2307,7 @@
       <c r="M19" s="24"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="33"/>
+      <c r="A20" s="34"/>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
       <c r="D20" s="28"/>
@@ -2322,7 +2322,7 @@
       <c r="M20" s="24"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="32">
+      <c r="A21" s="33">
         <v>9</v>
       </c>
       <c r="B21" s="24"/>
@@ -2339,7 +2339,7 @@
       <c r="M21" s="24"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="33"/>
+      <c r="A22" s="34"/>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
       <c r="D22" s="28"/>
@@ -2354,7 +2354,7 @@
       <c r="M22" s="24"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="32">
+      <c r="A23" s="33">
         <v>10</v>
       </c>
       <c r="B23" s="24"/>
@@ -2371,7 +2371,7 @@
       <c r="M23" s="24"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="33"/>
+      <c r="A24" s="34"/>
       <c r="B24" s="27"/>
       <c r="C24" s="27"/>
       <c r="D24" s="28"/>
@@ -2386,7 +2386,7 @@
       <c r="M24" s="24"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="32">
+      <c r="A25" s="33">
         <v>11</v>
       </c>
       <c r="B25" s="24"/>
@@ -2403,7 +2403,7 @@
       <c r="M25" s="24"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="33"/>
+      <c r="A26" s="34"/>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
       <c r="D26" s="28"/>
@@ -2418,7 +2418,7 @@
       <c r="M26" s="24"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="32">
+      <c r="A27" s="33">
         <v>12</v>
       </c>
       <c r="B27" s="24"/>
@@ -2435,7 +2435,7 @@
       <c r="M27" s="24"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" s="33"/>
+      <c r="A28" s="34"/>
       <c r="B28" s="27"/>
       <c r="C28" s="27"/>
       <c r="D28" s="28"/>
@@ -2450,7 +2450,7 @@
       <c r="M28" s="24"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="32">
+      <c r="A29" s="33">
         <v>13</v>
       </c>
       <c r="B29" s="24"/>
@@ -2467,7 +2467,7 @@
       <c r="M29" s="24"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" s="33"/>
+      <c r="A30" s="34"/>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
       <c r="D30" s="28"/>
@@ -2482,7 +2482,7 @@
       <c r="M30" s="24"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" s="32">
+      <c r="A31" s="33">
         <v>14</v>
       </c>
       <c r="B31" s="24"/>
@@ -2499,7 +2499,7 @@
       <c r="M31" s="24"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="33"/>
+      <c r="A32" s="34"/>
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
       <c r="D32" s="28"/>
@@ -2514,7 +2514,7 @@
       <c r="M32" s="24"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A33" s="32">
+      <c r="A33" s="33">
         <v>15</v>
       </c>
       <c r="B33" s="24"/>
@@ -2531,7 +2531,7 @@
       <c r="M33" s="24"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A34" s="33"/>
+      <c r="A34" s="34"/>
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
       <c r="D34" s="28"/>
@@ -2546,7 +2546,7 @@
       <c r="M34" s="24"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A35" s="32">
+      <c r="A35" s="33">
         <v>16</v>
       </c>
       <c r="B35" s="24"/>
@@ -2563,7 +2563,7 @@
       <c r="M35" s="24"/>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A36" s="33"/>
+      <c r="A36" s="34"/>
       <c r="B36" s="27"/>
       <c r="C36" s="27"/>
       <c r="D36" s="28"/>
@@ -2578,7 +2578,7 @@
       <c r="M36" s="24"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A37" s="32">
+      <c r="A37" s="33">
         <v>17</v>
       </c>
       <c r="B37" s="24"/>
@@ -2595,7 +2595,7 @@
       <c r="M37" s="24"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A38" s="33"/>
+      <c r="A38" s="34"/>
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
       <c r="D38" s="28"/>
@@ -2610,13 +2610,13 @@
       <c r="M38" s="24"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="36"/>
-      <c r="C39" s="36"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="37"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
       <c r="F39" s="31">
         <f>SUM(F5:F38)</f>
         <v>0</v>
@@ -2720,13 +2720,21 @@
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
     </row>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A1:M2"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
     <mergeCell ref="A31:A32"/>
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
@@ -2742,6 +2750,11 @@
     <mergeCell ref="A37:A38"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A1:M2"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>